<commit_message>
Atualização dos boletins e remoção de arquivos redundantes (29/07/2026)
</commit_message>
<xml_diff>
--- a/sources/2D_Manha_2_Bimestre.xlsx
+++ b/sources/2D_Manha_2_Bimestre.xlsx
@@ -61,7 +61,7 @@
     <x:t>Conselho Segundo Bimestre</x:t>
   </x:si>
   <x:si>
-    <x:t>318</x:t>
+    <x:t>320</x:t>
   </x:si>
   <x:si>
     <x:t>0 (Soma de todas as eletivas)</x:t>
@@ -247,163 +247,163 @@
     <x:t>15</x:t>
   </x:si>
   <x:si>
+    <x:t>78%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>86%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CHRISTIAN CARDOSO FERREIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMANUELY GUEDES BARROS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>99%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>98%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMELYN DOS SANTOS SANTANA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENZO GUIMARAES DA SILVA ARAUJO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESTHER CAROLINE PITA ALMEIDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EVILLYN VITÓRIA DOS ANJOS SANTOS SARAIVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEOVANNA TAVARES SANTANA BRAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>80%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GIOVANNA MELLANI SILVA RIBEIRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>87%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUILHERME GOMES DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HELOAH REBECA MONTEIRO DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>97%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISABELLA MOREIRA NOVAIS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>75%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>84%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISABELLY DE MELO MEIRA ANDRADE</x:t>
+  </x:si>
+  <x:si>
     <x:t>77%</x:t>
   </x:si>
   <x:si>
-    <x:t>86%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CHRISTIAN CARDOSO FERREIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMANUELY GUEDES BARROS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>99%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>98%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMELYN DOS SANTOS SANTANA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENZO GUIMARAES DA SILVA ARAUJO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESTHER CAROLINE PITA ALMEIDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EVILLYN VITÓRIA DOS ANJOS SANTOS SARAIVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEOVANNA TAVARES SANTANA BRAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>80%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GIOVANNA MELLANI SILVA RIBEIRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>87%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>90%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUILHERME GOMES DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>91%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HELOAH REBECA MONTEIRO DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISABELLA MOREIRA NOVAIS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>75%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>84%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISABELLY DE MELO MEIRA ANDRADE</x:t>
+    <x:t>JULIA BEATRIZ SILVA BORGES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>60%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>69%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JULIA EMANUELE RASSILAN LACERDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>82%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>85%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JULIA VALECK CIRINO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAMILLY VICTORIA SANTOS BAZARELLO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>79%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KEMILY VICENTE MATEUS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>48%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>61%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LAIS SOUZA NEGRI DO NASCIMENTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Não Comparecimento</x:t>
+  </x:si>
+  <x:si>
+    <x:t>72%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>74%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LETHICIA JESUS DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUCAS CASTANHEIRA SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARCELLA FRANCA ROMAO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARIA EDUARDA ALVES MATHIAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>67%</x:t>
   </x:si>
   <x:si>
     <x:t>76%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JULIA BEATRIZ SILVA BORGES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>59%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>69%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JULIA EMANUELE RASSILAN LACERDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>82%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>85%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JULIA VALECK CIRINO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>97%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAMILLY VICTORIA SANTOS BAZARELLO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>79%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KEMILY VICENTE MATEUS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>47%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>61%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LAIS SOUZA NEGRI DO NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Não Comparecimento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>72%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>73%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LETHICIA JESUS DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>78%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUCAS CASTANHEIRA SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARCELLA FRANCA ROMAO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARIA EDUARDA ALVES MATHIAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>66%</x:t>
   </x:si>
   <x:si>
     <x:t>MARIA VITÓRIA RODRIGUES DOS SANTOS</x:t>
@@ -1850,10 +1850,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW15" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX15" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY15" s="12">
         <x:v>0</x:v>
@@ -3505,7 +3505,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="BB25" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:54">
@@ -3707,7 +3707,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="L27" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="M27" s="12" t="s">
         <x:v>66</x:v>
@@ -3743,7 +3743,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="X27" s="12" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="Y27" s="12" t="s">
         <x:v>50</x:v>
@@ -3982,10 +3982,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW28" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX28" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY28" s="12">
         <x:v>0</x:v>
@@ -3997,12 +3997,12 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="BB28" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:54">
       <x:c r="A29" s="11" t="s">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B29" s="12" t="s">
         <x:v>45</x:v>
@@ -4026,7 +4026,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="I29" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="J29" s="12" t="s">
         <x:v>48</x:v>
@@ -4113,7 +4113,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AL29" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="AM29" s="12">
         <x:v>17</x:v>
@@ -4155,18 +4155,18 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="AZ29" s="12" t="s">
-        <x:v>96</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BA29" s="12">
         <x:v>97</x:v>
       </x:c>
       <x:c r="BB29" s="12" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:54">
       <x:c r="A30" s="11" t="s">
-        <x:v>98</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B30" s="12" t="s">
         <x:v>45</x:v>
@@ -4190,7 +4190,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="I30" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="J30" s="12" t="s">
         <x:v>48</x:v>
@@ -4319,7 +4319,7 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="AZ30" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="BA30" s="12">
         <x:v>100</x:v>
@@ -4330,7 +4330,7 @@
     </x:row>
     <x:row r="31" spans="1:54">
       <x:c r="A31" s="11" t="s">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="B31" s="12" t="s">
         <x:v>45</x:v>
@@ -4351,10 +4351,10 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="H31" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="I31" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="J31" s="12" t="s">
         <x:v>48</x:v>
@@ -4363,7 +4363,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="L31" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="M31" s="12" t="s">
         <x:v>49</x:v>
@@ -4414,7 +4414,7 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="AC31" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="AD31" s="12" t="s">
         <x:v>48</x:v>
@@ -4483,18 +4483,18 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="AZ31" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="BA31" s="12">
         <x:v>184</x:v>
       </x:c>
       <x:c r="BB31" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:54">
       <x:c r="A32" s="11" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B32" s="12" t="s">
         <x:v>45</x:v>
@@ -4605,7 +4605,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="AL32" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="AM32" s="12">
         <x:v>20</x:v>
@@ -4647,18 +4647,18 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="AZ32" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="BA32" s="12">
         <x:v>89</x:v>
       </x:c>
       <x:c r="BB32" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:54">
       <x:c r="A33" s="11" t="s">
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B33" s="12" t="s">
         <x:v>45</x:v>
@@ -4811,7 +4811,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="AZ33" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="BA33" s="12">
         <x:v>23</x:v>
@@ -4981,7 +4981,7 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="BB34" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:54">
@@ -5007,7 +5007,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="H35" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="I35" s="12" t="s">
         <x:v>112</x:v>
@@ -5019,7 +5019,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="L35" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="M35" s="12" t="s">
         <x:v>46</x:v>
@@ -5070,7 +5070,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AC35" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="AD35" s="12" t="s">
         <x:v>48</x:v>
@@ -5294,10 +5294,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW36" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX36" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY36" s="12">
         <x:v>88</x:v>
@@ -5458,10 +5458,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW37" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX37" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY37" s="12">
         <x:v>0</x:v>
@@ -5473,12 +5473,12 @@
         <x:v>125</x:v>
       </x:c>
       <x:c r="BB37" s="12" t="s">
-        <x:v>121</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:54">
       <x:c r="A38" s="11" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B38" s="12" t="s">
         <x:v>45</x:v>
@@ -5637,12 +5637,12 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="BB38" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:54">
       <x:c r="A39" s="11" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B39" s="12" t="s">
         <x:v>61</x:v>
@@ -5786,10 +5786,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW39" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX39" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY39" s="12">
         <x:v>0</x:v>
@@ -5806,7 +5806,7 @@
     </x:row>
     <x:row r="40" spans="1:54">
       <x:c r="A40" s="11" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B40" s="12" t="s">
         <x:v>45</x:v>
@@ -5917,7 +5917,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="AL40" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="AM40" s="12">
         <x:v>28</x:v>
@@ -5947,7 +5947,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="AV40" s="12" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AW40" s="12" t="s">
         <x:v>58</x:v>
@@ -5959,13 +5959,13 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="AZ40" s="12" t="s">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="BA40" s="12">
         <x:v>143</x:v>
       </x:c>
       <x:c r="BB40" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:54">
@@ -6129,7 +6129,7 @@
         <x:v>105</x:v>
       </x:c>
       <x:c r="BB41" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:54">
@@ -6278,10 +6278,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW42" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX42" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY42" s="12">
         <x:v>0</x:v>
@@ -7098,10 +7098,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW47" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX47" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY47" s="12">
         <x:v>0</x:v>
@@ -7113,7 +7113,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="BB47" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:54">
@@ -7751,7 +7751,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="AV51" s="12" t="s">
-        <x:v>47</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="AW51" s="12" t="s">
         <x:v>58</x:v>
@@ -7769,7 +7769,7 @@
         <x:v>108</x:v>
       </x:c>
       <x:c r="BB51" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:54">
@@ -7915,7 +7915,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="AV52" s="12" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AW52" s="12" t="s">
         <x:v>50</x:v>
@@ -8246,10 +8246,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="AW54" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AX54" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AY54" s="12">
         <x:v>0</x:v>
@@ -8261,7 +8261,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="BB54" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:54">
@@ -8583,7 +8583,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AZ56" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BA56" s="12">
         <x:v>71</x:v>
@@ -8988,7 +8988,7 @@
       <x:c r="AO59" s="7"/>
       <x:c r="AP59" s="7"/>
       <x:c r="AQ59" s="7" t="s">
-        <x:v>151</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="AR59" s="7"/>
       <x:c r="AS59" s="7"/>

</xml_diff>